<commit_message>
📊 Horarios actualizados Línea 141 - 5068
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-10-12.xlsx
+++ b/data/horarios-141-2026-10-12.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:01:34</t>
+          <t>Última actualización: 14:45:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 13</t>
+          <t>Total filas: 19</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>05:01:34</t>
+          <t>14:45:47</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>05:17</t>
+          <t>14:45</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>05:01:34</t>
+          <t>14:45:47</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>05:22</t>
+          <t>14:54</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>05:01:34</t>
+          <t>14:45:47</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>05:44</t>
+          <t>15:01</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>43</v>
+        <v>16</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>05:01:34</t>
+          <t>14:45:47</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>05:47</t>
+          <t>15:04</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>46</v>
+        <v>19</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,12 +573,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>05:01:34</t>
+          <t>14:45:47</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>06:01</t>
+          <t>15:06</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -587,7 +587,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>60</v>
+        <v>21</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,21 +598,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>05:01:34</t>
+          <t>14:45:47</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>06:09</t>
+          <t>15:15</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>68</v>
+        <v>30</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,21 +623,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>05:01:34</t>
+          <t>14:45:47</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06:12</t>
+          <t>15:24</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>71</v>
+        <v>39</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -648,21 +648,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>05:01:34</t>
+          <t>14:45:47</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>15:34</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>89</v>
+        <v>49</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,21 +673,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>05:01:34</t>
+          <t>14:45:47</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>06:36</t>
+          <t>15:41</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>95</v>
+        <v>56</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -698,21 +698,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>05:01:34</t>
+          <t>14:45:47</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>06:39</t>
+          <t>15:44</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>98</v>
+        <v>59</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -723,21 +723,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>05:01:34</t>
+          <t>14:45:47</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>06:41</t>
+          <t>15:55</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,21 +748,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>05:01:34</t>
+          <t>14:45:47</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>06:41</t>
+          <t>15:56</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>100</v>
+        <v>71</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -773,23 +773,173 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>05:01:34</t>
+          <t>14:45:47</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>06:59</t>
+          <t>16:01</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>76</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>14:45:47</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>16:04</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>79</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>14:45:47</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>16:14</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>89</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>14:45:47</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>16:24</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>99</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>14:45:47</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>16:34</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>109</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>14:45:47</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>16:35</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>110</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>14:45:47</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>16:44</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
           <t>225_GOMEZ</t>
         </is>
       </c>
-      <c r="D18" t="n">
-        <v>118</v>
-      </c>
-      <c r="E18" t="inlineStr">
+      <c r="D24" t="n">
+        <v>119</v>
+      </c>
+      <c r="E24" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -806,7 +956,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -819,14 +969,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:01:34</t>
+          <t>Última actualización: 14:45:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -860,23 +1010,73 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>05:01:34</t>
+          <t>14:45:47</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>06:12</t>
+          <t>14:54</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>71</v>
+        <v>9</v>
       </c>
       <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>14:45:47</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>15:04</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>19</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>14:45:47</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>15:34</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>49</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -893,7 +1093,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -906,14 +1106,116 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:01:34</t>
+          <t>Última actualización: 14:45:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>14:45:47</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>15:22</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>37</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>14:45:47</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>16:02</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>77</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>14:45:47</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>16:29</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>104</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 5069
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-10-12.xlsx
+++ b/data/horarios-141-2026-10-12.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:45:47</t>
+          <t>Última actualización: 20:46:17</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 19</t>
+          <t>Total filas: 33</t>
         </is>
       </c>
     </row>
@@ -940,6 +940,356 @@
         <v>119</v>
       </c>
       <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>20:46:17</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>20:51</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>5</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>20:46:17</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>20:57</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>11</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>20:46:17</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>21:06</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>20</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>20:46:17</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>21:06</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>20</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>20:46:17</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>21:34</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>48</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>20:46:17</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>21:36</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>50</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>20:46:17</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>21:37</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>51</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>20:46:17</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>21:49</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>63</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>20:46:17</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>21:59</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>73</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>20:46:17</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>21:59</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>73</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>20:46:17</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>22:07</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>81</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>20:46:17</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>22:26</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>100</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>20:46:17</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>22:37</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>111</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>20:46:17</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>22:41</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>115</v>
+      </c>
+      <c r="E38" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -956,7 +1306,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -969,14 +1319,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:45:47</t>
+          <t>Última actualización: 20:46:17</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 6</t>
         </is>
       </c>
     </row>
@@ -1077,6 +1427,81 @@
         <v>49</v>
       </c>
       <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>20:46:17</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>21:06</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>20</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>20:46:17</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>21:59</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>73</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>20:46:17</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>22:37</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>111</v>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1093,7 +1518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1106,14 +1531,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:45:47</t>
+          <t>Última actualización: 20:46:17</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 4</t>
         </is>
       </c>
     </row>
@@ -1216,6 +1641,31 @@
       <c r="E8" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>20:46:17</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>21:32</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>46</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>